<commit_message>
Organize docs and harden DGX live run workflow
</commit_message>
<xml_diff>
--- a/excels/test_suite_template.xlsx
+++ b/excels/test_suite_template.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Case_Index" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Case_Steps" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Test_Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Run_Config" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Dictionary" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Case_Index - 用例索引" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Case_Steps - 用例步骤" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Test_Data - 测试数据" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Run_Config - 运行配置" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Dictionary - 字典配置" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="中文说明" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -50,8 +51,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -126,6 +130,361 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DGXTest</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>用例唯一标识，例如 DGX_001。</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>用例名称，建议写业务可读标题。</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>一级模块，例如 DGX。</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>二级模块，例如 Demo。</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>功能点名称。</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>用例类型，例如 functional。</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>优先级，例如 P1 / P2。</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>测试层级，例如 smoke。</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>标签，多个值用英文逗号分隔。</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>用例状态，例如 active。</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>是否自动化，Y/N。</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>前置条件编号，可为空。</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>前置条件说明。</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>后置条件说明，可为空。</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>关联测试数据集 ID。</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>环境范围，多个值用英文逗号分隔。</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>浏览器范围，多个值用英文逗号分隔。</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>是否允许并行，Y/N。</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>失败重试策略标识。</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>责任人。</t>
+      </text>
+    </comment>
+    <comment ref="U1" authorId="0" shapeId="0">
+      <text>
+        <t>是否要求先登录，Y/N。</t>
+      </text>
+    </comment>
+    <comment ref="V1" authorId="0" shapeId="0">
+      <text>
+        <t>依赖的前置用例 ID，可为空。</t>
+      </text>
+    </comment>
+    <comment ref="W1" authorId="0" shapeId="0">
+      <text>
+        <t>期望结果摘要。</t>
+      </text>
+    </comment>
+    <comment ref="X1" authorId="0" shapeId="0">
+      <text>
+        <t>给 AI 的额外提示。</t>
+      </text>
+    </comment>
+    <comment ref="Y1" authorId="0" shapeId="0">
+      <text>
+        <t>备注说明。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DGXTest</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>所属用例 ID。</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>步骤序号，从 1 开始。</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>步骤类型，常见为 action / assert。</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>步骤名称，建议写成业务动作。</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>动作关键字，例如 click、open_page。</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>断言关键字，例如 assert_text_contains（断言）。</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>所属页面对象名。</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>目标对象 key；如果是 open_page，可填写路由。</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>目标类型，例如 element / route。</t>
+      </text>
+    </comment>
+    <comment ref="J1" authorId="0" shapeId="0">
+      <text>
+        <t>输入值或动作值。</t>
+      </text>
+    </comment>
+    <comment ref="K1" authorId="0" shapeId="0">
+      <text>
+        <t>值类型，例如 string。</t>
+      </text>
+    </comment>
+    <comment ref="L1" authorId="0" shapeId="0">
+      <text>
+        <t>期望结果，例如 expected（期望结果）可写断言文本。</t>
+      </text>
+    </comment>
+    <comment ref="M1" authorId="0" shapeId="0">
+      <text>
+        <t>期望值类型，例如 string。</t>
+      </text>
+    </comment>
+    <comment ref="N1" authorId="0" shapeId="0">
+      <text>
+        <t>匹配方式，例如 contains / equals。</t>
+      </text>
+    </comment>
+    <comment ref="O1" authorId="0" shapeId="0">
+      <text>
+        <t>等待策略，例如 visible / dom_ready。</t>
+      </text>
+    </comment>
+    <comment ref="P1" authorId="0" shapeId="0">
+      <text>
+        <t>超时时间，单位秒。</t>
+      </text>
+    </comment>
+    <comment ref="Q1" authorId="0" shapeId="0">
+      <text>
+        <t>失败后是否继续，Y/N。</t>
+      </text>
+    </comment>
+    <comment ref="R1" authorId="0" shapeId="0">
+      <text>
+        <t>失败时是否截图，Y/N。</t>
+      </text>
+    </comment>
+    <comment ref="S1" authorId="0" shapeId="0">
+      <text>
+        <t>给 AI 或定位器的提示。</t>
+      </text>
+    </comment>
+    <comment ref="T1" authorId="0" shapeId="0">
+      <text>
+        <t>步骤备注。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DGXTest</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>数据集唯一 ID。</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>数据集名称。</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>所属模块。</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>使用环境。</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>示例业务字段：项目名。</t>
+      </text>
+    </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>示例业务字段：结果区域项目名。</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>示例业务字段：图层选项。</t>
+      </text>
+    </comment>
+    <comment ref="H1" authorId="0" shapeId="0">
+      <text>
+        <t>备注。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DGXTest</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>配置键。</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>配置值。</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>备注。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment5.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>DGXTest</author>
+  </authors>
+  <commentList>
+    <comment ref="A1" authorId="0" shapeId="0">
+      <text>
+        <t>字典类型。</t>
+      </text>
+    </comment>
+    <comment ref="B1" authorId="0" shapeId="0">
+      <text>
+        <t>字典值。</t>
+      </text>
+    </comment>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>字典中文含义或展示名。</t>
+      </text>
+    </comment>
+    <comment ref="D1" authorId="0" shapeId="0">
+      <text>
+        <t>是否启用，Y/N。</t>
+      </text>
+    </comment>
+    <comment ref="E1" authorId="0" shapeId="0">
+      <text>
+        <t>备注。</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -412,138 +771,163 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>case_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>case_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>module</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>sub_module</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>feature_name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>case_type</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>test_level</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>tags</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>status</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>automation_flag</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>precondition_id</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>preconditions</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>postconditions</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>data_set_id</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>env_scope</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>browser_scope</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>can_parallel</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>retry_policy</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>owner</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>require_login</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>depends_on_case</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>expected_result_summary</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>ai_hint</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>remark</t>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>case_id
+用例ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>case_name
+用例名称</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>module
+模块</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>sub_module
+子模块</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>feature_name
+功能点</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>case_type
+用例类型</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>priority
+优先级</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>test_level
+测试层级</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>tags
+标签</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>status
+状态</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>automation_flag
+自动化标记</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>precondition_id
+前置条件ID</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>preconditions
+前置条件</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>postconditions
+后置条件</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>data_set_id
+数据集ID</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>env_scope
+环境范围</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>browser_scope
+浏览器范围</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>can_parallel
+是否并行</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>retry_policy
+重试策略</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>owner
+负责人</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>require_login
+是否需要登录</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>depends_on_case
+依赖用例</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>expected_result_summary
+期望结果摘要</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>ai_hint
+AI提示</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>remark
+备注</t>
         </is>
       </c>
     </row>
@@ -777,119 +1161,255 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DGX_003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Verify DGX landing page stable entry state</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>DGX</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Demo</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Landing Smoke</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>functional</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>dgx,demo,landing</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Demo URL is reachable</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>DATA_DGX_DEFAULT_01</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>demo</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>chromium</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>case_retry_1</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>tester</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>Landing page keeps the expected route and entry controls visible</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>Fast smoke case focused on the DGX landing entry state</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>Default DGX landing regression case</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T29"/>
+  <dimension ref="A1:T36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>case_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>step_no</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>step_type</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>step_name</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>action_key</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>assert_key</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>page_name</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>target</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>target_type</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
-        <is>
-          <t>value_type</t>
-        </is>
-      </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>expected</t>
-        </is>
-      </c>
-      <c r="M1" t="inlineStr">
-        <is>
-          <t>expected_type</t>
-        </is>
-      </c>
-      <c r="N1" t="inlineStr">
-        <is>
-          <t>match_type</t>
-        </is>
-      </c>
-      <c r="O1" t="inlineStr">
-        <is>
-          <t>wait</t>
-        </is>
-      </c>
-      <c r="P1" t="inlineStr">
-        <is>
-          <t>timeout</t>
-        </is>
-      </c>
-      <c r="Q1" t="inlineStr">
-        <is>
-          <t>continue_on_fail</t>
-        </is>
-      </c>
-      <c r="R1" t="inlineStr">
-        <is>
-          <t>screenshot_on_fail</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>ai_locator_hint</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>remark</t>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>case_id
+用例ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>step_no
+步骤序号</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>step_type
+步骤类型</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>step_name
+步骤名称</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>action_key
+动作关键字</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>assert_key
+断言关键字</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>page_name
+页面名</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>target
+目标对象</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>target_type
+目标类型</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>value
+输入值</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>value_type
+值类型</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>expected
+期望结果</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>expected_type
+期望类型</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>match_type
+匹配方式</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>wait
+等待策略</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>timeout
+超时秒数</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>continue_on_fail
+失败后继续</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>screenshot_on_fail
+失败截图</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>ai_locator_hint
+定位提示</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>remark
+备注</t>
         </is>
       </c>
     </row>
@@ -970,45 +1490,49 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>assert</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Open project card entry button</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>Assert DGX demo route</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>assert_url_equals</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>DGXLandingPage</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>project_card_entry_button</t>
-        </is>
-      </c>
+      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>route</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>visible</t>
-        </is>
-      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>https://dgx.xlook.ai/dgx/f2b850f5-14a0-4325-b56d-cb1213f63ec2</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>10</v>
       </c>
@@ -1022,12 +1546,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>Faya entry button</t>
-        </is>
-      </c>
-      <c r="T3" t="inlineStr"/>
+      <c r="S3" t="inlineStr"/>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Assert the landing page opens the exact recorded DGX demo route</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1045,7 +1569,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Enter project workspace</t>
+          <t>Open project card entry button</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1061,7 +1585,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>project_go_to_button</t>
+          <t>project_card_entry_button</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -1094,7 +1618,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Go to project</t>
+          <t>Faya entry button</t>
         </is>
       </c>
       <c r="T4" t="inlineStr"/>
@@ -1110,29 +1634,45 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>assert</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Assert project workspace opened (placeholder)</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>Enter project workspace</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>DGXLandingPage</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>project_go_to_button</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
       <c r="P5" t="n">
         <v>10</v>
       </c>
@@ -1146,12 +1686,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S5" t="inlineStr"/>
-      <c r="T5" t="inlineStr">
-        <is>
-          <t>Assertion placeholder: fill assert_key, target, expected, and match_type later. Empty placeholder assertions are skipped by the runner.</t>
-        </is>
-      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>Go to project</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1164,23 +1704,23 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>assert</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Open Set Boundaries panel</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>Assert project workspace opened</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>DGXBoundaryPage</t>
+          <t>DGXLandingPage</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -1218,10 +1758,14 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Set Boundaries</t>
-        </is>
-      </c>
-      <c r="T6" t="inlineStr"/>
+          <t>Workspace entry ready</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>Assert workspace loaded by checking Set Boundaries entry is visible</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1234,29 +1778,45 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>assert</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Assert Set Boundaries panel opened (placeholder)</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>Open Set Boundaries panel</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>set_boundaries_button</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr"/>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
       <c r="P7" t="n">
         <v>10</v>
       </c>
@@ -1270,12 +1830,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr">
-        <is>
-          <t>Assertion placeholder: fill assert_key, target, expected, and match_type later. Empty placeholder assertions are skipped by the runner.</t>
-        </is>
-      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>Set Boundaries</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1293,13 +1853,13 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Verify upload entry is visible</t>
+          <t>Assert Set Boundaries panel opened</t>
         </is>
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
-          <t>assert_text_contains</t>
+          <t>assert_element_visible</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1319,21 +1879,9 @@
       </c>
       <c r="J8" t="inlineStr"/>
       <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>UploadPlot CAD File</t>
-        </is>
-      </c>
-      <c r="M8" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>contains</t>
-        </is>
-      </c>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
       <c r="O8" t="inlineStr">
         <is>
           <t>visible</t>
@@ -1357,16 +1905,20 @@
           <t>UploadPlot CAD File</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>Assert the boundary panel exposes the upload entry</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DGX_002</t>
+          <t>DGX_001</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1375,28 +1927,28 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Open DGX demo landing page</t>
+          <t>Wait upload entry is visible</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>open_page</t>
+          <t>wait_element</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
-          <t>DGXLandingPage</t>
+          <t>DGXBoundaryPage</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>/dgx/f2b850f5-14a0-4325-b56d-cb1213f63ec2</t>
+          <t>upload_plot_button</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>route</t>
+          <t>element</t>
         </is>
       </c>
       <c r="J9" t="inlineStr"/>
@@ -1406,7 +1958,7 @@
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr">
         <is>
-          <t>dom_ready</t>
+          <t>visible</t>
         </is>
       </c>
       <c r="P9" t="n">
@@ -1422,8 +1974,16 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>UploadPlot CAD File</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>Wait until the upload entry is stably visible before leaving the panel</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1432,7 +1992,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1441,12 +2001,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Open project card entry button</t>
+          <t>Open DGX demo landing page</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>click</t>
+          <t>open_page</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1457,12 +2017,12 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>project_card_entry_button</t>
+          <t>/dgx/f2b850f5-14a0-4325-b56d-cb1213f63ec2</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>route</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -1472,7 +2032,7 @@
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr">
         <is>
-          <t>visible</t>
+          <t>dom_ready</t>
         </is>
       </c>
       <c r="P10" t="n">
@@ -1488,11 +2048,7 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S10" t="inlineStr">
-        <is>
-          <t>Faya entry button</t>
-        </is>
-      </c>
+      <c r="S10" t="inlineStr"/>
       <c r="T10" t="inlineStr"/>
     </row>
     <row r="11">
@@ -1502,49 +2058,53 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>assert</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Enter project workspace</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>Assert DGX demo route</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>assert_url_equals</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>DGXLandingPage</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>project_go_to_button</t>
-        </is>
-      </c>
+      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>route</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>visible</t>
-        </is>
-      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>https://dgx.xlook.ai/dgx/f2b850f5-14a0-4325-b56d-cb1213f63ec2</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>10</v>
       </c>
@@ -1558,12 +2118,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S11" t="inlineStr">
-        <is>
-          <t>Go to project</t>
-        </is>
-      </c>
-      <c r="T11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>Assert the landing page opens the exact recorded DGX demo route</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1572,7 +2132,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1581,7 +2141,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Open Set Boundaries panel</t>
+          <t>Open project card entry button</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -1592,12 +2152,12 @@
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
-          <t>DGXBoundaryPage</t>
+          <t>DGXLandingPage</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>set_boundaries_button</t>
+          <t>project_card_entry_button</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1630,7 +2190,7 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Set Boundaries</t>
+          <t>Faya entry button</t>
         </is>
       </c>
       <c r="T12" t="inlineStr"/>
@@ -1642,7 +2202,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1651,7 +2211,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Open plot upload dialog</t>
+          <t>Enter project workspace</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -1662,12 +2222,12 @@
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>DGXBoundaryPage</t>
+          <t>DGXLandingPage</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>upload_plot_button</t>
+          <t>project_go_to_button</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1700,7 +2260,7 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>UploadPlot CAD File</t>
+          <t>Go to project</t>
         </is>
       </c>
       <c r="T13" t="inlineStr"/>
@@ -1712,33 +2272,49 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>assert</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Assert upload dialog opened (placeholder)</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>Open Set Boundaries panel</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>set_boundaries_button</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
       <c r="P14" t="n">
         <v>10</v>
       </c>
@@ -1752,12 +2328,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr">
-        <is>
-          <t>Assertion placeholder: fill assert_key, target, expected, and match_type later. Empty placeholder assertions are skipped by the runner.</t>
-        </is>
-      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Set Boundaries</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1766,7 +2342,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1775,7 +2351,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Open first layer selector</t>
+          <t>Open plot upload dialog</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -1791,7 +2367,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>layer_select_button_1</t>
+          <t>upload_plot_button</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1824,7 +2400,7 @@
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>First layer selector</t>
+          <t>UploadPlot CAD File</t>
         </is>
       </c>
       <c r="T15" t="inlineStr"/>
@@ -1836,24 +2412,24 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>assert</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Choose Not Required for first layer</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>Assert upload dialog opened</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
@@ -1861,7 +2437,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>not_required_option</t>
+          <t>layer_select_button_1</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -1894,10 +2470,14 @@
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>Not Required option</t>
-        </is>
-      </c>
-      <c r="T16" t="inlineStr"/>
+          <t>First layer selector</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>Assert the upload dialog shows the layer selector</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1906,7 +2486,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1915,7 +2495,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Open second layer selector</t>
+          <t>Open first layer selector</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -1931,7 +2511,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>layer_select_button_2</t>
+          <t>layer_select_button_1</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1964,7 +2544,7 @@
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>Second layer selector</t>
+          <t>First layer selector</t>
         </is>
       </c>
       <c r="T17" t="inlineStr"/>
@@ -1976,7 +2556,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1985,7 +2565,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Choose Not Required for second layer</t>
+          <t>Choose Not Required for first layer</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -2046,7 +2626,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -2055,7 +2635,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Close upload dialog</t>
+          <t>Open second layer selector</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -2071,7 +2651,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>cancel_button</t>
+          <t>layer_select_button_2</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -2104,7 +2684,7 @@
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>Cancel button</t>
+          <t>Second layer selector</t>
         </is>
       </c>
       <c r="T19" t="inlineStr"/>
@@ -2116,7 +2696,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2125,7 +2705,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Go to next setup step</t>
+          <t>Choose Not Required for second layer</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -2141,7 +2721,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>next_button</t>
+          <t>not_required_option</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -2174,7 +2754,7 @@
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>Next button</t>
+          <t>Not Required option</t>
         </is>
       </c>
       <c r="T20" t="inlineStr"/>
@@ -2186,33 +2766,49 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>assert</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Assert layer visibility step opened (placeholder)</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr"/>
+          <t>Close upload dialog</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>cancel_button</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
       <c r="P21" t="n">
         <v>10</v>
       </c>
@@ -2226,12 +2822,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S21" t="inlineStr"/>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>Assertion placeholder: fill assert_key, target, expected, and match_type later. Empty placeholder assertions are skipped by the runner.</t>
-        </is>
-      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Cancel button</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2240,24 +2836,24 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>assert</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Go to layer visibility step</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>click</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
+          <t>Assert upload dialog closed</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>assert_element_hidden</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
@@ -2265,7 +2861,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>next_button</t>
+          <t>layer_select_button_1</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -2280,7 +2876,7 @@
       <c r="N22" t="inlineStr"/>
       <c r="O22" t="inlineStr">
         <is>
-          <t>visible</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="P22" t="n">
@@ -2298,10 +2894,14 @@
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>Next button</t>
-        </is>
-      </c>
-      <c r="T22" t="inlineStr"/>
+          <t>First layer selector</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Assert the upload dialog is gone before moving to the next footer step</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2310,7 +2910,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2319,12 +2919,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hide all layers</t>
+          <t>Go to next setup step</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>uncheck</t>
+          <t>click</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -2335,7 +2935,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>show_hide_all_checkbox</t>
+          <t>next_button</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2368,7 +2968,7 @@
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>Show Hide All checkbox</t>
+          <t>Next button</t>
         </is>
       </c>
       <c r="T23" t="inlineStr"/>
@@ -2380,24 +2980,24 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>assert</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Enable first layer</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>check</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+          <t>Assert layer visibility step opened</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
@@ -2405,7 +3005,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>layer_checkbox_1</t>
+          <t>plot_area_assignment_active_label</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -2438,10 +3038,14 @@
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>First layer checkbox</t>
-        </is>
-      </c>
-      <c r="T24" t="inlineStr"/>
+          <t>Active boundary step label</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Assert the first footer Next moved into Plot Area Assignment</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2450,7 +3054,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2459,12 +3063,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Enable second layer</t>
+          <t>Go to layer visibility step</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>click</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -2475,7 +3079,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>layer_checkbox_2</t>
+          <t>next_button</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -2508,7 +3112,7 @@
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>Second layer checkbox</t>
+          <t>Next button</t>
         </is>
       </c>
       <c r="T25" t="inlineStr"/>
@@ -2520,7 +3124,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2529,12 +3133,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Show all layers</t>
+          <t>Hide all layers</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>uncheck</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -2590,7 +3194,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2599,12 +3203,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Finish boundary setup</t>
+          <t>Enable first layer</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>click</t>
+          <t>check</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -2615,7 +3219,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>done_button</t>
+          <t>layer_checkbox_1</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -2648,7 +3252,7 @@
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>Done button</t>
+          <t>First layer checkbox</t>
         </is>
       </c>
       <c r="T27" t="inlineStr"/>
@@ -2660,33 +3264,49 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>assert</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Assert design result area updated (placeholder)</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr"/>
+          <t>Enable second layer</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
       <c r="F28" t="inlineStr"/>
       <c r="G28" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
-      <c r="I28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>layer_checkbox_2</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
       <c r="J28" t="inlineStr"/>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
       <c r="P28" t="n">
         <v>10</v>
       </c>
@@ -2700,12 +3320,12 @@
           <t>Y</t>
         </is>
       </c>
-      <c r="S28" t="inlineStr"/>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>Assertion placeholder: fill assert_key, target, expected, and match_type later. Empty placeholder assertions are skipped by the runner.</t>
-        </is>
-      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Second layer checkbox</t>
+        </is>
+      </c>
+      <c r="T28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2714,24 +3334,24 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>assert</t>
+          <t>action</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Verify result project cell</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr"/>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>assert_text_contains</t>
-        </is>
-      </c>
+          <t>Show all layers</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>DGXBoundaryPage</t>
@@ -2739,7 +3359,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>project_result_cell</t>
+          <t>show_hide_all_checkbox</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -2749,21 +3369,9 @@
       </c>
       <c r="J29" t="inlineStr"/>
       <c r="K29" t="inlineStr"/>
-      <c r="L29" t="inlineStr">
-        <is>
-          <t>${project_result_name}</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr">
-        <is>
-          <t>string</t>
-        </is>
-      </c>
-      <c r="N29" t="inlineStr">
-        <is>
-          <t>contains</t>
-        </is>
-      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr"/>
+      <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr">
         <is>
           <t>visible</t>
@@ -2784,18 +3392,537 @@
       </c>
       <c r="S29" t="inlineStr">
         <is>
+          <t>Show Hide All checkbox</t>
+        </is>
+      </c>
+      <c r="T29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DGX_002</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>21</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Finish boundary setup</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr"/>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>DGXBoundaryPage</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>done_button</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr"/>
+      <c r="M30" t="inlineStr"/>
+      <c r="N30" t="inlineStr"/>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P30" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R30" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Done button</t>
+        </is>
+      </c>
+      <c r="T30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>DGX_002</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>22</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Wait design result area updated</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>wait_element</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr"/>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>DGXBoundaryPage</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>project_result_cell</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr"/>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr"/>
+      <c r="M31" t="inlineStr"/>
+      <c r="N31" t="inlineStr"/>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
           <t>Project result cell</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>Wait until the result area is visible before checking the project name</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>DGX_002</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>23</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Verify result project cell</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>assert_text_equals</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>DGXBoundaryPage</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>project_result_cell</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr"/>
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>${project_result_name}</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Project result cell</t>
+        </is>
+      </c>
+      <c r="T32" t="inlineStr">
+        <is>
+          <t>Assert the result area shows the exact expected project after Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>DGX_003</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Open DGX demo landing page</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>open_page</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>DGXLandingPage</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>/dgx/f2b850f5-14a0-4325-b56d-cb1213f63ec2</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr"/>
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr"/>
+      <c r="N33" t="inlineStr"/>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>dom_ready</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S33" t="inlineStr"/>
+      <c r="T33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DGX_003</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>2</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Assert DGX demo route</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>assert_url_equals</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>DGXLandingPage</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>route</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr"/>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://dgx.xlook.ai/dgx/f2b850f5-14a0-4325-b56d-cb1213f63ec2</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>equals</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr"/>
+      <c r="P34" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S34" t="inlineStr"/>
+      <c r="T34" t="inlineStr">
+        <is>
+          <t>Assert the landing page opens the exact recorded DGX demo route</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>DGX_003</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>3</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Open project card entry button</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>DGXLandingPage</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>project_card_entry_button</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr"/>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr"/>
+      <c r="N35" t="inlineStr"/>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Faya entry button</t>
+        </is>
+      </c>
+      <c r="T35" t="inlineStr">
+        <is>
+          <t>Open the landing project card before asserting the Go to Configuration control</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DGX_003</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>4</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Assert go to button visible</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr"/>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>DGXLandingPage</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>project_go_to_button</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>element</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr"/>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr"/>
+      <c r="N36" t="inlineStr"/>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>visible</t>
+        </is>
+      </c>
+      <c r="P36" t="n">
+        <v>10</v>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="S36" t="inlineStr">
+        <is>
+          <t>Go to project</t>
+        </is>
+      </c>
+      <c r="T36" t="inlineStr">
+        <is>
+          <t>Assert the DGX landing page exposes the Go to Configuration button after opening the project card</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2803,45 +3930,53 @@
   <dimension ref="A1:H2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>data_set_id</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>data_name</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>module</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>env</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>project_name</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>project_result_name</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>layer_option</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>remark</t>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>data_set_id
+数据集ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>data_name
+数据集名称</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>module
+模块</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>env
+环境</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>project_name
+项目名称</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>project_result_name
+结果项目名</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>layer_option
+图层选项</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>remark
+备注</t>
         </is>
       </c>
     </row>
@@ -2889,11 +4024,12 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
@@ -2901,20 +4037,23 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>config_key</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>config_value</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>remark</t>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>config_key
+配置键</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>config_value
+配置值</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>remark
+备注</t>
         </is>
       </c>
     </row>
@@ -2988,251 +4127,922 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="anysvml"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dict_type
+字典类型</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>dict_value
+字典值</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dict_label
+字典标签</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>enabled
+是否启用</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>remark
+备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>priority</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>test_level</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>smoke</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Smoke</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>status</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>open_page</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Open page</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>click</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Click</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>clear_and_input</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Clear and input</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>input_password</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Input password</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>input_text</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Input text</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>check</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>uncheck</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Uncheck</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>wait_element</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Wait element</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>select_option</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Select option</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>action_key</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>upload_file</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Upload file</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>assert_url_contains</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Assert URL contains</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>assert_url_equals</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Assert URL equals</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>assert_element_visible</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Assert element visible</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>assert_element_hidden</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Assert element hidden</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>assert_text_contains</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Assert text contains</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>assert_text_equals</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Assert text equals</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>assert_value_equals</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Assert value equals</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>dict_type</t>
+          <t>类别</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>dict_value</t>
+          <t>英文名</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>dict_label</t>
+          <t>中文说明</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>remark</t>
+          <t>补充说明</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>priority</t>
+          <t>说明</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>parser_compatibility</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>兼容性说明</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>priority</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>P2</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>请勿修改双语表头中的英文第一行关键字；代码解析时以英文关键字为准。中文仅用于阅读辅助。</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>test_level</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>smoke</t>
+          <t>sheet_name</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Smoke</t>
+          <t>中文名称</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr"/>
+          <t>说明</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>status</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>active</t>
+          <t>Case_Index</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>用例索引</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr"/>
+          <t>工作表 Case_Index = 用例索引</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>action_key</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>open_page</t>
+          <t>Case_Steps</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Open page</t>
+          <t>用例步骤</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr"/>
+          <t>工作表 Case_Steps = 用例步骤</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>action_key</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>click</t>
+          <t>Test_Data</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Click</t>
+          <t>测试数据</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr"/>
+          <t>工作表 Test_Data = 测试数据</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>action_key</t>
+          <t>Sheet</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>check</t>
+          <t>Run_Config</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>运行配置</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr"/>
+          <t>工作表 Run_Config = 运行配置</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Dictionary</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>字典配置</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>工作表 Dictionary = 字典配置</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>english_key</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>中文含义</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>说明</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>action</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>动作步骤</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>执行点击、输入、勾选等操作。</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>assert</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>断言步骤</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>用于校验页面状态或文本是否符合预期。</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>expected</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>期望结果</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>断言时希望看到的文本、URL 或结果。</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>assert_key</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>断言关键字</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>例如 assert_text_contains，表示断言方式。</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>action_key</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>uncheck</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Uncheck</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>assert_key</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>assert_text_contains</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Assert text contains</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>动作关键字</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>例如 click、open_page、check。</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>target</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>目标对象</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>步骤实际操作或断言的对象 key。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>object_key</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>对象库主键</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>对象库里的唯一标识，会被步骤 target 引用。</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>字段</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>remark</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>备注</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>补充说明，不参与核心执行逻辑。</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>